<commit_message>
Version usando llama3 con Ollama (local)
</commit_message>
<xml_diff>
--- a/Casos de Regatas.xlsx
+++ b/Casos de Regatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/Inteligencia Artificial Aplicada/Materias/04. Procesamiento de Lenguaje Natural/TP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/Inteligencia Artificial Aplicada/Materias/04. Procesamiento de Lenguaje Natural/DIIA-PLN-TP-Final/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="94" documentId="11_2C447A9E1C490587C5EB8AD627D4F21B5C78B259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3196FA3D-900A-CA43-8597-A93AD75CEBA2}"/>
   <bookViews>
-    <workbookView xWindow="34100" yWindow="2200" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="300" yWindow="880" windowWidth="34540" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos de Regatas y sus Títulos" sheetId="1" r:id="rId1"/>
@@ -1572,10 +1572,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Ajustado el System Prompt para CoT, para ver si con tunning se obtienen mejores respuestas. También se agregaron los ejemplos para los prompts de la estrategia FS CoT
</commit_message>
<xml_diff>
--- a/Casos de Regatas.xlsx
+++ b/Casos de Regatas.xlsx
@@ -1,26 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10406"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/Inteligencia Artificial Aplicada/Materias/04. Procesamiento de Lenguaje Natural/DIIA-PLN-TP-Final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/01. Inteligencia Artificial Aplicada/Materias/04. Procesamiento de Lenguaje Natural/99. DIIA-PLN-TP-Final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="11_2C447A9E1C490587C5EB8AD627D4F21B5C78B259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3196FA3D-900A-CA43-8597-A93AD75CEBA2}"/>
+  <xr:revisionPtr revIDLastSave="271" documentId="11_2C447A9E1C490587C5EB8AD627D4F21B5C78B259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D593CC31-402B-2B4B-B0DA-6A9493322C0C}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="880" windowWidth="34540" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33680" yWindow="1940" windowWidth="33660" windowHeight="17360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos de Regatas y sus Títulos" sheetId="1" r:id="rId1"/>
+    <sheet name="Resultados" sheetId="2" r:id="rId2"/>
+    <sheet name="Análisis" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="71">
   <si>
     <t>ID</t>
   </si>
@@ -1457,13 +1472,80 @@
       </rPr>
       <t>: Penalizar a B.</t>
     </r>
+  </si>
+  <si>
+    <t>Prompt Español</t>
+  </si>
+  <si>
+    <t>Prompt inglés</t>
+  </si>
+  <si>
+    <t>Chain-of-Thought (CoT)</t>
+  </si>
+  <si>
+    <t>Few-Shot 
+Chain-of-Thought (FS CoT)</t>
+  </si>
+  <si>
+    <t>Comentarios</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>Falla</t>
+  </si>
+  <si>
+    <t>CoT - ES: El resultado es correcto, pero el modelo alucina en el rationale y en la regla aplicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoT - ES: Solo aplica la regla 11 pero no aplica la regla 16.1 </t>
+  </si>
+  <si>
+    <t>CoT - EN:</t>
+  </si>
+  <si>
+    <t>FS CoT - ES:</t>
+  </si>
+  <si>
+    <t>FS CoT - EN:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoT - ES: </t>
+  </si>
+  <si>
+    <t>CoT - ES: Alucina en el rationale y con las reglas</t>
+  </si>
+  <si>
+    <t>CoT - ES: El modelo interpreta el escenario de manera particular (asume que el barco B completó la virada)</t>
+  </si>
+  <si>
+    <t>CoT - ES: No explicita todas las reglas que deberían considerarse</t>
+  </si>
+  <si>
+    <t>CoT - ES: El modelo asume que el barco Y vira y choca</t>
+  </si>
+  <si>
+    <t>CoT - ES: Las reglas mencionadas no se ajustan al Ground Thruth</t>
+  </si>
+  <si>
+    <t>CoT - ES: Identifica bien la regla, pero interpreta mal los puntos de aplicación</t>
+  </si>
+  <si>
+    <t>CoT - ES: El modelo asume que B choca, y toma la decisión correcta penalizando. La reglas de aplicación tienen sentido</t>
+  </si>
+  <si>
+    <t>CoT - ES: El análisis de modelo es correcto, pero hay una "zona gris" del escenario que probablemente causa confusión</t>
+  </si>
+  <si>
+    <t>CoT - ES: Razonamiento incorrecto</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1500,6 +1582,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1515,7 +1603,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1538,11 +1626,130 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1557,9 +1764,77 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2011,4 +2286,812 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17CDA499-0016-9E48-AD79-F5B2F70F2B84}">
+  <dimension ref="A1:G64"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="85.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="A1" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="G3" s="12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B4" s="11"/>
+      <c r="C4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B6" s="15"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B7" s="15"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B8" s="16"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B9" s="14">
+        <v>2</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="27" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B10" s="15"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B11" s="15"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B13" s="14">
+        <v>3</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="27" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B14" s="15"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B15" s="15"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="28" x14ac:dyDescent="0.15">
+      <c r="B17" s="14">
+        <v>4</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B18" s="15"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B19" s="15"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B20" s="16"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B21" s="19">
+        <v>5</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B22" s="20"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B23" s="20"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B24" s="21"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B25" s="19">
+        <v>6</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="27" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B26" s="20"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B27" s="20"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B28" s="23"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B29" s="24">
+        <v>7</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B30" s="20"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B31" s="20"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B32" s="23"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B33" s="24">
+        <v>8</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="27" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B34" s="20"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B35" s="20"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B36" s="23"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" ht="28" x14ac:dyDescent="0.15">
+      <c r="B37" s="24">
+        <v>9</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="27" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B38" s="20"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B39" s="20"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B40" s="23"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" ht="28" x14ac:dyDescent="0.15">
+      <c r="B41" s="24">
+        <v>10</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B42" s="20"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B43" s="20"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B44" s="23"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B45" s="24">
+        <v>11</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="27" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B46" s="20"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B47" s="20"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B48" s="23"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B49" s="24">
+        <v>12</v>
+      </c>
+      <c r="C49" s="17"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B50" s="20"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B51" s="20"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B52" s="23"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B53" s="24">
+        <v>13</v>
+      </c>
+      <c r="C53" s="17"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B54" s="20"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B55" s="20"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B56" s="23"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B57" s="24">
+        <v>14</v>
+      </c>
+      <c r="C57" s="17"/>
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B58" s="20"/>
+      <c r="C58" s="17"/>
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B59" s="20"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B60" s="23"/>
+      <c r="C60" s="17"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B61" s="24">
+        <v>15</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B62" s="20"/>
+      <c r="C62" s="17"/>
+      <c r="D62" s="22"/>
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B63" s="20"/>
+      <c r="C63" s="17"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" ht="14" x14ac:dyDescent="0.15">
+      <c r="B64" s="23"/>
+      <c r="C64" s="17"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="79">
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="F5:F8"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="B57:B60"/>
+    <mergeCell ref="C57:C60"/>
+    <mergeCell ref="D57:D60"/>
+    <mergeCell ref="E57:E60"/>
+    <mergeCell ref="F57:F60"/>
+    <mergeCell ref="B61:B64"/>
+    <mergeCell ref="C61:C64"/>
+    <mergeCell ref="D61:D64"/>
+    <mergeCell ref="E61:E64"/>
+    <mergeCell ref="F61:F64"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="C49:C52"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="E49:E52"/>
+    <mergeCell ref="F49:F52"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="E53:E56"/>
+    <mergeCell ref="F53:F56"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="C41:C44"/>
+    <mergeCell ref="D41:D44"/>
+    <mergeCell ref="E41:E44"/>
+    <mergeCell ref="F41:F44"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="C45:C48"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="E45:E48"/>
+    <mergeCell ref="F45:F48"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="C33:C36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E36"/>
+    <mergeCell ref="F33:F36"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="C37:C40"/>
+    <mergeCell ref="D37:D40"/>
+    <mergeCell ref="E37:E40"/>
+    <mergeCell ref="F37:F40"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="F25:F28"/>
+    <mergeCell ref="B29:B32"/>
+    <mergeCell ref="C29:C32"/>
+    <mergeCell ref="D29:D32"/>
+    <mergeCell ref="E29:E32"/>
+    <mergeCell ref="F29:F32"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="D17:D20"/>
+    <mergeCell ref="E17:E20"/>
+    <mergeCell ref="F17:F20"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="C21:C24"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="E21:E24"/>
+    <mergeCell ref="F21:F24"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="C13:C16"/>
+    <mergeCell ref="D13:D16"/>
+    <mergeCell ref="E13:E16"/>
+    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="B5:B8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED012409-1330-4547-82DA-5BA50D4F7AB8}">
+  <dimension ref="E6:K13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="6" spans="5:11" x14ac:dyDescent="0.15">
+      <c r="E6" s="28">
+        <f>COUNTIF(Resultados!C$5:C$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F6" s="28">
+        <f>COUNTIF(Resultados!C$5:C$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="13" spans="5:11" x14ac:dyDescent="0.15">
+      <c r="K13" s="28"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>